<commit_message>
Fix duplicate sentence in identity reliability intro a0da28eece91fd32819a39a167cb0fc6d3fe6685
</commit_message>
<xml_diff>
--- a/fix/298-identity-reliability-mandatory/ig/StructureDefinition-fr-core-identity-reliability.xlsx
+++ b/fix/298-identity-reliability-mandatory/ig/StructureDefinition-fr-core-identity-reliability.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-29T12:37:34+00:00</t>
+    <t>2026-10-07T07:07:43+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -491,7 +491,7 @@
     <t>Annotations complémentaires sur l’identité : attributs RNIV (homonyme, douteux, fictif) et codes de gestion (doublon, collision, désactivé…). Plusieurs annotations peuvent coexister.</t>
   </si>
   <si>
-    <t>En particulier, les attributs Identité douteuse (DOUT) et Identité fictive (FICT), combinés au statut Identité provisoire (PROV) imposé par les invariants ci-dessous, permettent de qualifier les cas où l'absence de vérification n'est pas une simple attente mais un problème identifié (homonymie non résolue, identité fictive ou anonyme, patient refusant de s'identifier...) : toute situation d'identitovigilance reste ainsi représentable. | In particular, the Doubtful identity (DOUT) and Fictitious identity (FICT) attributes, combined with the mandatory Provisional identity (PROV) status required by the invariants below, make it possible to qualify cases where the lack of verification is not a mere pending state but an identified issue (unresolved homonymy, fictitious or anonymous identity, patient refusing to be identified...): every identity vigilance situation remains representable this way.</t>
+    <t>En particulier, les attributs Identité douteuse (DOUT) et Identité fictive (FICT), combinés au statut Identité provisoire (PROV) imposé par les invariants ci-dessous, permettent d'indiquer les cas où l'absence de vérification n'est pas une simple attente mais un problème identifié (homonymie non résolue, identité fictive ou anonyme, patient refusant de s'identifier...) : toute situation d'identitovigilance reste ainsi représentable. | In particular, the Doubtful identity (DOUT) and Fictitious identity (FICT) attributes, combined with the mandatory Provisional identity (PROV) status required by the invariants below, make it possible to indicate cases where the lack of verification is not a mere pending state but an identified issue (unresolved homonymy, fictitious or anonymous identity, patient refusing to be identified...): every identity vigilance situation remains representable this way.</t>
   </si>
   <si>
     <t>Extension.extension:comment.id</t>

</xml_diff>